<commit_message>
Keep large reconciliation explanations responsive without weakening reference boundaries
</commit_message>
<xml_diff>
--- a/audit/assistant-evidence/browser-local/p5-partial-source-direct.xlsx
+++ b/audit/assistant-evidence/browser-local/p5-partial-source-direct.xlsx
@@ -1696,7 +1696,7 @@
     </row>
     <row r="2" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
-        <v>46295.82323171296</v>
+        <v>46295.8319477662</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>183</v>
@@ -2358,7 +2358,7 @@
         <v>250</v>
       </c>
       <c r="B5" s="4">
-        <v>46295.82323637731</v>
+        <v>46295.831952430555</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>